<commit_message>
Refactor dataset_detector and main modules to improve import structure and enhance profile detection functionality
</commit_message>
<xml_diff>
--- a/data/input/Entry.xlsx
+++ b/data/input/Entry.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\IT\Projects\Crd Smart Grouping\data\input\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5E9BFE4-46BB-428B-861F-0AB3AD1CAC33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-28920" yWindow="3015" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -2932,8 +2938,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2996,6 +3002,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -3042,7 +3056,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -3074,9 +3088,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -3108,6 +3140,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -3283,11 +3333,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M161"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3328,7 +3378,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -3366,7 +3416,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -3401,7 +3451,7 @@
         <v>990784</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -3436,7 +3486,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -3474,7 +3524,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -3512,7 +3562,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -3544,7 +3594,7 @@
         <v>463603</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -3585,7 +3635,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -3617,7 +3667,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -3625,7 +3675,7 @@
         <v>18</v>
       </c>
       <c r="C10">
-        <v>317.66</v>
+        <v>317.66000000000003</v>
       </c>
       <c r="D10" t="s">
         <v>38</v>
@@ -3655,7 +3705,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -3663,7 +3713,7 @@
         <v>18</v>
       </c>
       <c r="C11">
-        <v>317.66</v>
+        <v>317.66000000000003</v>
       </c>
       <c r="D11" t="s">
         <v>40</v>
@@ -3696,7 +3746,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -3728,7 +3778,7 @@
         <v>850578</v>
       </c>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -3766,7 +3816,7 @@
         <v>920</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -3774,7 +3824,7 @@
         <v>18</v>
       </c>
       <c r="C14">
-        <v>294.35</v>
+        <v>294.35000000000002</v>
       </c>
       <c r="D14" t="s">
         <v>39</v>
@@ -3804,7 +3854,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -3812,7 +3862,7 @@
         <v>18</v>
       </c>
       <c r="C15">
-        <v>294.35</v>
+        <v>294.35000000000002</v>
       </c>
       <c r="D15" t="s">
         <v>37</v>
@@ -3839,7 +3889,7 @@
         <v>922</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -3874,7 +3924,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -3909,7 +3959,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -3950,7 +4000,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -3991,7 +4041,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>13</v>
       </c>
@@ -4026,7 +4076,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -4064,7 +4114,7 @@
         <v>388629</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -4102,7 +4152,7 @@
         <v>764842</v>
       </c>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>14</v>
       </c>
@@ -4137,7 +4187,7 @@
         <v>994452</v>
       </c>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>13</v>
       </c>
@@ -4172,7 +4222,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>14</v>
       </c>
@@ -4210,7 +4260,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>13</v>
       </c>
@@ -4248,7 +4298,7 @@
         <v>766466</v>
       </c>
     </row>
-    <row r="27" spans="1:13">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>14</v>
       </c>
@@ -4283,7 +4333,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>13</v>
       </c>
@@ -4291,7 +4341,7 @@
         <v>18</v>
       </c>
       <c r="C28">
-        <v>88.54000000000001</v>
+        <v>88.54</v>
       </c>
       <c r="D28" t="s">
         <v>38</v>
@@ -4321,7 +4371,7 @@
         <v>824452</v>
       </c>
     </row>
-    <row r="29" spans="1:13">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>14</v>
       </c>
@@ -4329,7 +4379,7 @@
         <v>18</v>
       </c>
       <c r="C29">
-        <v>88.54000000000001</v>
+        <v>88.54</v>
       </c>
       <c r="D29" t="s">
         <v>40</v>
@@ -4356,7 +4406,7 @@
         <v>310191</v>
       </c>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>13</v>
       </c>
@@ -4397,7 +4447,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>14</v>
       </c>
@@ -4432,7 +4482,7 @@
         <v>928</v>
       </c>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>13</v>
       </c>
@@ -4470,7 +4520,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>14</v>
       </c>
@@ -4508,7 +4558,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="34" spans="1:13">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -4546,7 +4596,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>14</v>
       </c>
@@ -4584,7 +4634,7 @@
         <v>121433</v>
       </c>
     </row>
-    <row r="36" spans="1:13">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>13</v>
       </c>
@@ -4592,7 +4642,7 @@
         <v>17</v>
       </c>
       <c r="C36">
-        <v>91.31999999999999</v>
+        <v>91.32</v>
       </c>
       <c r="D36" t="s">
         <v>39</v>
@@ -4619,7 +4669,7 @@
         <v>805056</v>
       </c>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>14</v>
       </c>
@@ -4627,7 +4677,7 @@
         <v>17</v>
       </c>
       <c r="C37">
-        <v>91.31999999999999</v>
+        <v>91.32</v>
       </c>
       <c r="D37" t="s">
         <v>39</v>
@@ -4660,7 +4710,7 @@
         <v>931</v>
       </c>
     </row>
-    <row r="38" spans="1:13">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -4695,7 +4745,7 @@
         <v>344020</v>
       </c>
     </row>
-    <row r="39" spans="1:13">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>14</v>
       </c>
@@ -4736,7 +4786,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="40" spans="1:13">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -4774,7 +4824,7 @@
         <v>932</v>
       </c>
     </row>
-    <row r="41" spans="1:13">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>14</v>
       </c>
@@ -4812,7 +4862,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:13">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>14</v>
       </c>
@@ -4847,7 +4897,7 @@
         <v>741701</v>
       </c>
     </row>
-    <row r="43" spans="1:13">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>13</v>
       </c>
@@ -4888,7 +4938,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="44" spans="1:13">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>13</v>
       </c>
@@ -4926,7 +4976,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="45" spans="1:13">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>13</v>
       </c>
@@ -4961,7 +5011,7 @@
         <v>799156</v>
       </c>
     </row>
-    <row r="46" spans="1:13">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>14</v>
       </c>
@@ -4999,7 +5049,7 @@
         <v>994155</v>
       </c>
     </row>
-    <row r="47" spans="1:13">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>13</v>
       </c>
@@ -5007,7 +5057,7 @@
         <v>18</v>
       </c>
       <c r="C47">
-        <v>85.56999999999999</v>
+        <v>85.57</v>
       </c>
       <c r="D47" t="s">
         <v>40</v>
@@ -5040,7 +5090,7 @@
         <v>423549</v>
       </c>
     </row>
-    <row r="48" spans="1:13">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>13</v>
       </c>
@@ -5078,7 +5128,7 @@
         <v>396587</v>
       </c>
     </row>
-    <row r="49" spans="1:13">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>13</v>
       </c>
@@ -5110,7 +5160,7 @@
         <v>667482</v>
       </c>
     </row>
-    <row r="50" spans="1:13">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>14</v>
       </c>
@@ -5142,7 +5192,7 @@
         <v>36402</v>
       </c>
     </row>
-    <row r="51" spans="1:13">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>13</v>
       </c>
@@ -5177,7 +5227,7 @@
         <v>935</v>
       </c>
     </row>
-    <row r="52" spans="1:13">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>13</v>
       </c>
@@ -5185,7 +5235,7 @@
         <v>17</v>
       </c>
       <c r="C52">
-        <v>71.09999999999999</v>
+        <v>71.099999999999994</v>
       </c>
       <c r="D52" t="s">
         <v>40</v>
@@ -5218,7 +5268,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="53" spans="1:13">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>13</v>
       </c>
@@ -5226,7 +5276,7 @@
         <v>17</v>
       </c>
       <c r="C53">
-        <v>35.55</v>
+        <v>35.549999999999997</v>
       </c>
       <c r="D53" t="s">
         <v>37</v>
@@ -5253,7 +5303,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="54" spans="1:13">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>14</v>
       </c>
@@ -5288,7 +5338,7 @@
         <v>10308</v>
       </c>
     </row>
-    <row r="55" spans="1:13">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>13</v>
       </c>
@@ -5320,7 +5370,7 @@
         <v>938</v>
       </c>
     </row>
-    <row r="56" spans="1:13">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>13</v>
       </c>
@@ -5328,7 +5378,7 @@
         <v>17</v>
       </c>
       <c r="C56">
-        <v>85.65000000000001</v>
+        <v>85.65</v>
       </c>
       <c r="D56" t="s">
         <v>38</v>
@@ -5355,7 +5405,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="57" spans="1:13">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>13</v>
       </c>
@@ -5390,7 +5440,7 @@
         <v>400277</v>
       </c>
     </row>
-    <row r="58" spans="1:13">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>14</v>
       </c>
@@ -5398,7 +5448,7 @@
         <v>18</v>
       </c>
       <c r="C58">
-        <v>284.91</v>
+        <v>284.91000000000003</v>
       </c>
       <c r="D58" t="s">
         <v>39</v>
@@ -5428,7 +5478,7 @@
         <v>445283</v>
       </c>
     </row>
-    <row r="59" spans="1:13">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>13</v>
       </c>
@@ -5460,7 +5510,7 @@
         <v>940</v>
       </c>
     </row>
-    <row r="60" spans="1:13">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>13</v>
       </c>
@@ -5495,7 +5545,7 @@
         <v>179742</v>
       </c>
     </row>
-    <row r="61" spans="1:13">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>13</v>
       </c>
@@ -5533,7 +5583,7 @@
         <v>836923</v>
       </c>
     </row>
-    <row r="62" spans="1:13">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>14</v>
       </c>
@@ -5571,7 +5621,7 @@
         <v>291173</v>
       </c>
     </row>
-    <row r="63" spans="1:13">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>13</v>
       </c>
@@ -5606,7 +5656,7 @@
         <v>950133</v>
       </c>
     </row>
-    <row r="64" spans="1:13">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>13</v>
       </c>
@@ -5644,7 +5694,7 @@
         <v>941</v>
       </c>
     </row>
-    <row r="65" spans="1:13">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>13</v>
       </c>
@@ -5682,7 +5732,7 @@
         <v>690436</v>
       </c>
     </row>
-    <row r="66" spans="1:13">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>14</v>
       </c>
@@ -5720,7 +5770,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="67" spans="1:13">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>13</v>
       </c>
@@ -5758,7 +5808,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="68" spans="1:13">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>13</v>
       </c>
@@ -5799,7 +5849,7 @@
         <v>41482</v>
       </c>
     </row>
-    <row r="69" spans="1:13">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>13</v>
       </c>
@@ -5834,7 +5884,7 @@
         <v>151823</v>
       </c>
     </row>
-    <row r="70" spans="1:13">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>14</v>
       </c>
@@ -5872,7 +5922,7 @@
         <v>655880</v>
       </c>
     </row>
-    <row r="71" spans="1:13">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>13</v>
       </c>
@@ -5910,7 +5960,7 @@
         <v>310584</v>
       </c>
     </row>
-    <row r="72" spans="1:13">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>13</v>
       </c>
@@ -5948,7 +5998,7 @@
         <v>646632</v>
       </c>
     </row>
-    <row r="73" spans="1:13">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>13</v>
       </c>
@@ -5986,7 +6036,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="74" spans="1:13">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>14</v>
       </c>
@@ -6024,7 +6074,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="75" spans="1:13">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>13</v>
       </c>
@@ -6056,7 +6106,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="76" spans="1:13">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>13</v>
       </c>
@@ -6097,7 +6147,7 @@
         <v>943</v>
       </c>
     </row>
-    <row r="77" spans="1:13">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>13</v>
       </c>
@@ -6105,7 +6155,7 @@
         <v>17</v>
       </c>
       <c r="C77">
-        <v>77.70999999999999</v>
+        <v>77.709999999999994</v>
       </c>
       <c r="D77" t="s">
         <v>39</v>
@@ -6132,7 +6182,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="78" spans="1:13">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>14</v>
       </c>
@@ -6167,7 +6217,7 @@
         <v>874890</v>
       </c>
     </row>
-    <row r="79" spans="1:13">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>13</v>
       </c>
@@ -6208,7 +6258,7 @@
         <v>944</v>
       </c>
     </row>
-    <row r="80" spans="1:13">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>13</v>
       </c>
@@ -6216,7 +6266,7 @@
         <v>17</v>
       </c>
       <c r="C80">
-        <v>72.40000000000001</v>
+        <v>72.400000000000006</v>
       </c>
       <c r="D80" t="s">
         <v>38</v>
@@ -6237,7 +6287,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="81" spans="1:13">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>13</v>
       </c>
@@ -6245,7 +6295,7 @@
         <v>17</v>
       </c>
       <c r="C81">
-        <v>36.2</v>
+        <v>36.200000000000003</v>
       </c>
       <c r="D81" t="s">
         <v>39</v>
@@ -6278,7 +6328,7 @@
         <v>999189</v>
       </c>
     </row>
-    <row r="82" spans="1:13">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>13</v>
       </c>
@@ -6319,7 +6369,7 @@
         <v>695935</v>
       </c>
     </row>
-    <row r="83" spans="1:13">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>14</v>
       </c>
@@ -6354,7 +6404,7 @@
         <v>179199</v>
       </c>
     </row>
-    <row r="84" spans="1:13">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>13</v>
       </c>
@@ -6392,7 +6442,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="85" spans="1:13">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>14</v>
       </c>
@@ -6427,7 +6477,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="86" spans="1:13">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>13</v>
       </c>
@@ -6462,7 +6512,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="87" spans="1:13">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>14</v>
       </c>
@@ -6491,7 +6541,7 @@
         <v>352591</v>
       </c>
     </row>
-    <row r="88" spans="1:13">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>13</v>
       </c>
@@ -6532,7 +6582,7 @@
         <v>437204</v>
       </c>
     </row>
-    <row r="89" spans="1:13">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>14</v>
       </c>
@@ -6567,7 +6617,7 @@
         <v>772372</v>
       </c>
     </row>
-    <row r="90" spans="1:13">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>13</v>
       </c>
@@ -6602,7 +6652,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="91" spans="1:13">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>14</v>
       </c>
@@ -6610,7 +6660,7 @@
         <v>17</v>
       </c>
       <c r="C91">
-        <v>134.77</v>
+        <v>134.77000000000001</v>
       </c>
       <c r="D91" t="s">
         <v>39</v>
@@ -6643,7 +6693,7 @@
         <v>948</v>
       </c>
     </row>
-    <row r="92" spans="1:13">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>13</v>
       </c>
@@ -6678,7 +6728,7 @@
         <v>441032</v>
       </c>
     </row>
-    <row r="93" spans="1:13">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>14</v>
       </c>
@@ -6716,7 +6766,7 @@
         <v>931279</v>
       </c>
     </row>
-    <row r="94" spans="1:13">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>13</v>
       </c>
@@ -6751,7 +6801,7 @@
         <v>949</v>
       </c>
     </row>
-    <row r="95" spans="1:13">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>14</v>
       </c>
@@ -6786,7 +6836,7 @@
         <v>865771</v>
       </c>
     </row>
-    <row r="96" spans="1:13">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>13</v>
       </c>
@@ -6824,7 +6874,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="97" spans="1:13">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>14</v>
       </c>
@@ -6862,7 +6912,7 @@
         <v>597131</v>
       </c>
     </row>
-    <row r="98" spans="1:13">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>13</v>
       </c>
@@ -6903,7 +6953,7 @@
         <v>319041</v>
       </c>
     </row>
-    <row r="99" spans="1:13">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>14</v>
       </c>
@@ -6941,7 +6991,7 @@
         <v>302875</v>
       </c>
     </row>
-    <row r="100" spans="1:13">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>13</v>
       </c>
@@ -6979,7 +7029,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="101" spans="1:13">
+    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>14</v>
       </c>
@@ -7017,7 +7067,7 @@
         <v>952</v>
       </c>
     </row>
-    <row r="102" spans="1:13">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>13</v>
       </c>
@@ -7025,7 +7075,7 @@
         <v>18</v>
       </c>
       <c r="C102">
-        <v>572.5599999999999</v>
+        <v>572.55999999999995</v>
       </c>
       <c r="D102" t="s">
         <v>39</v>
@@ -7052,7 +7102,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="103" spans="1:13">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>13</v>
       </c>
@@ -7090,7 +7140,7 @@
         <v>164482</v>
       </c>
     </row>
-    <row r="104" spans="1:13">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>13</v>
       </c>
@@ -7128,7 +7178,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="105" spans="1:13">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>15</v>
       </c>
@@ -7163,7 +7213,7 @@
         <v>641649</v>
       </c>
     </row>
-    <row r="106" spans="1:13">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>15</v>
       </c>
@@ -7201,7 +7251,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="107" spans="1:13">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>15</v>
       </c>
@@ -7209,7 +7259,7 @@
         <v>18</v>
       </c>
       <c r="C107">
-        <v>539.9400000000001</v>
+        <v>539.94000000000005</v>
       </c>
       <c r="D107" t="s">
         <v>38</v>
@@ -7236,7 +7286,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="108" spans="1:13">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>15</v>
       </c>
@@ -7277,7 +7327,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="109" spans="1:13">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>16</v>
       </c>
@@ -7312,7 +7362,7 @@
         <v>956</v>
       </c>
     </row>
-    <row r="110" spans="1:13">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>15</v>
       </c>
@@ -7344,7 +7394,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="111" spans="1:13">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>13</v>
       </c>
@@ -7379,7 +7429,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="112" spans="1:13">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>14</v>
       </c>
@@ -7414,7 +7464,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="113" spans="1:13">
+    <row r="113" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>14</v>
       </c>
@@ -7455,7 +7505,7 @@
         <v>935132</v>
       </c>
     </row>
-    <row r="114" spans="1:13">
+    <row r="114" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>15</v>
       </c>
@@ -7493,7 +7543,7 @@
         <v>364270</v>
       </c>
     </row>
-    <row r="115" spans="1:13">
+    <row r="115" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>14</v>
       </c>
@@ -7528,7 +7578,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="116" spans="1:13">
+    <row r="116" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>15</v>
       </c>
@@ -7563,7 +7613,7 @@
         <v>991844</v>
       </c>
     </row>
-    <row r="117" spans="1:13">
+    <row r="117" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>14</v>
       </c>
@@ -7601,7 +7651,7 @@
         <v>848980</v>
       </c>
     </row>
-    <row r="118" spans="1:13">
+    <row r="118" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>15</v>
       </c>
@@ -7636,7 +7686,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="119" spans="1:13">
+    <row r="119" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>13</v>
       </c>
@@ -7674,7 +7724,7 @@
         <v>643540</v>
       </c>
     </row>
-    <row r="120" spans="1:13">
+    <row r="120" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>16</v>
       </c>
@@ -7715,7 +7765,7 @@
         <v>300010</v>
       </c>
     </row>
-    <row r="121" spans="1:13">
+    <row r="121" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>13</v>
       </c>
@@ -7750,7 +7800,7 @@
         <v>685233</v>
       </c>
     </row>
-    <row r="122" spans="1:13">
+    <row r="122" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>15</v>
       </c>
@@ -7788,7 +7838,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="123" spans="1:13">
+    <row r="123" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>14</v>
       </c>
@@ -7826,7 +7876,7 @@
         <v>959</v>
       </c>
     </row>
-    <row r="124" spans="1:13">
+    <row r="124" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>15</v>
       </c>
@@ -7864,7 +7914,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="125" spans="1:13">
+    <row r="125" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>15</v>
       </c>
@@ -7902,7 +7952,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="126" spans="1:13">
+    <row r="126" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>16</v>
       </c>
@@ -7943,7 +7993,7 @@
         <v>962</v>
       </c>
     </row>
-    <row r="127" spans="1:13">
+    <row r="127" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>15</v>
       </c>
@@ -7978,7 +8028,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="128" spans="1:13">
+    <row r="128" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>13</v>
       </c>
@@ -8016,7 +8066,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="129" spans="1:13">
+    <row r="129" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>15</v>
       </c>
@@ -8051,7 +8101,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="130" spans="1:13">
+    <row r="130" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>16</v>
       </c>
@@ -8092,7 +8142,7 @@
         <v>611041</v>
       </c>
     </row>
-    <row r="131" spans="1:13">
+    <row r="131" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>15</v>
       </c>
@@ -8124,7 +8174,7 @@
         <v>944757</v>
       </c>
     </row>
-    <row r="132" spans="1:13">
+    <row r="132" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>15</v>
       </c>
@@ -8159,7 +8209,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="133" spans="1:13">
+    <row r="133" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>15</v>
       </c>
@@ -8167,7 +8217,7 @@
         <v>18</v>
       </c>
       <c r="C133">
-        <v>159.8</v>
+        <v>159.80000000000001</v>
       </c>
       <c r="D133" t="s">
         <v>39</v>
@@ -8200,7 +8250,7 @@
         <v>145643</v>
       </c>
     </row>
-    <row r="134" spans="1:13">
+    <row r="134" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>14</v>
       </c>
@@ -8238,7 +8288,7 @@
         <v>965</v>
       </c>
     </row>
-    <row r="135" spans="1:13">
+    <row r="135" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>16</v>
       </c>
@@ -8276,7 +8326,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="136" spans="1:13">
+    <row r="136" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>15</v>
       </c>
@@ -8317,7 +8367,7 @@
         <v>358501</v>
       </c>
     </row>
-    <row r="137" spans="1:13">
+    <row r="137" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>14</v>
       </c>
@@ -8349,7 +8399,7 @@
         <v>949384</v>
       </c>
     </row>
-    <row r="138" spans="1:13">
+    <row r="138" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>14</v>
       </c>
@@ -8387,7 +8437,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="139" spans="1:13">
+    <row r="139" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>16</v>
       </c>
@@ -8425,7 +8475,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="140" spans="1:13">
+    <row r="140" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>13</v>
       </c>
@@ -8463,7 +8513,7 @@
         <v>651038</v>
       </c>
     </row>
-    <row r="141" spans="1:13">
+    <row r="141" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>13</v>
       </c>
@@ -8498,7 +8548,7 @@
         <v>967</v>
       </c>
     </row>
-    <row r="142" spans="1:13">
+    <row r="142" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>14</v>
       </c>
@@ -8506,7 +8556,7 @@
         <v>18</v>
       </c>
       <c r="C142">
-        <v>18.17</v>
+        <v>18.170000000000002</v>
       </c>
       <c r="D142" t="s">
         <v>37</v>
@@ -8536,7 +8586,7 @@
         <v>896499</v>
       </c>
     </row>
-    <row r="143" spans="1:13">
+    <row r="143" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>13</v>
       </c>
@@ -8544,7 +8594,7 @@
         <v>17</v>
       </c>
       <c r="C143">
-        <v>132.64</v>
+        <v>132.63999999999999</v>
       </c>
       <c r="D143" t="s">
         <v>39</v>
@@ -8571,7 +8621,7 @@
         <v>97950</v>
       </c>
     </row>
-    <row r="144" spans="1:13">
+    <row r="144" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>13</v>
       </c>
@@ -8609,7 +8659,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="145" spans="1:13">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>14</v>
       </c>
@@ -8647,7 +8697,7 @@
         <v>834431</v>
       </c>
     </row>
-    <row r="146" spans="1:13">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>13</v>
       </c>
@@ -8682,7 +8732,7 @@
         <v>427055</v>
       </c>
     </row>
-    <row r="147" spans="1:13">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>14</v>
       </c>
@@ -8720,7 +8770,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="148" spans="1:13">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>16</v>
       </c>
@@ -8758,7 +8808,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="149" spans="1:13">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>13</v>
       </c>
@@ -8787,7 +8837,7 @@
         <v>886390</v>
       </c>
     </row>
-    <row r="150" spans="1:13">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>14</v>
       </c>
@@ -8825,7 +8875,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="151" spans="1:13">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>16</v>
       </c>
@@ -8863,7 +8913,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="152" spans="1:13">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>14</v>
       </c>
@@ -8895,7 +8945,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="153" spans="1:13">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>13</v>
       </c>
@@ -8930,7 +8980,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="154" spans="1:13">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>14</v>
       </c>
@@ -8968,7 +9018,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="155" spans="1:13">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>15</v>
       </c>
@@ -8976,7 +9026,7 @@
         <v>18</v>
       </c>
       <c r="C155">
-        <v>683.1799999999999</v>
+        <v>683.18</v>
       </c>
       <c r="D155" t="s">
         <v>38</v>
@@ -9003,7 +9053,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="156" spans="1:13">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>14</v>
       </c>
@@ -9041,7 +9091,7 @@
         <v>970</v>
       </c>
     </row>
-    <row r="157" spans="1:13">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>13</v>
       </c>
@@ -9079,7 +9129,7 @@
         <v>100238</v>
       </c>
     </row>
-    <row r="158" spans="1:13">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>13</v>
       </c>
@@ -9111,7 +9161,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="159" spans="1:13">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>13</v>
       </c>
@@ -9146,7 +9196,7 @@
         <v>338551</v>
       </c>
     </row>
-    <row r="160" spans="1:13">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>13</v>
       </c>
@@ -9184,7 +9234,7 @@
         <v>73404</v>
       </c>
     </row>
-    <row r="161" spans="1:13">
+    <row r="161" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>16</v>
       </c>

</xml_diff>